<commit_message>
Corrección en los excel resumen
</commit_message>
<xml_diff>
--- a/http/resultados mediciones/resumen_brutos_http.xlsx
+++ b/http/resultados mediciones/resumen_brutos_http.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\angel\Desktop\TFG\local\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\angel\Desktop\TFG\Repositorio\Desarrollo-de-practicas-con-unikernels\http\resultados mediciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{557E9E3C-7AB0-4FAE-8017-50667EEE0D23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FBD3394-5EE3-43E3-B074-71CFCC1FA20E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20610" yWindow="-1155" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6885" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6883" uniqueCount="249">
   <si>
     <t>Resumen de resultados HTTP (R1–R10)</t>
   </si>
@@ -784,12 +784,6 @@
     <t>TotalMiB calculado</t>
   </si>
   <si>
-    <t>TotalMiB del CSV</t>
-  </si>
-  <si>
-    <t>Diferencia</t>
-  </si>
-  <si>
     <t>tamanos_desplegables.csv</t>
   </si>
 </sst>
@@ -55409,31 +55403,27 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A2:F8"/>
+  <dimension ref="A2:D8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="32" customWidth="1"/>
+    <col min="4" max="4" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" ht="15.6">
+    <row r="2" spans="1:4" ht="15.6">
       <c r="A2" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="14.4">
+    <row r="3" spans="1:4" ht="14.4">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-    </row>
-    <row r="5" spans="1:6" ht="25.95" customHeight="1">
+    </row>
+    <row r="5" spans="1:4" ht="25.95" customHeight="1" thickBot="1">
       <c r="A5" s="4" t="s">
         <v>2</v>
       </c>
@@ -55444,16 +55434,10 @@
         <v>247</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>248</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="F5" s="4" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:4" ht="14.4" thickBot="1">
       <c r="A6" s="5" t="s">
         <v>7</v>
       </c>
@@ -55464,18 +55448,11 @@
         <f>B6/1048576</f>
         <v>7.0015392303466797</v>
       </c>
-      <c r="D6" s="7">
-        <v>7.0019999999999998</v>
-      </c>
-      <c r="E6" s="7">
-        <f>ROUND(C6-D6,3)</f>
-        <v>0</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
+      <c r="D6" s="5" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="14.4" thickBot="1">
       <c r="A7" s="5" t="s">
         <v>8</v>
       </c>
@@ -55486,18 +55463,11 @@
         <f>B7/1048576</f>
         <v>2.2515392303466797</v>
       </c>
-      <c r="D7" s="7">
-        <v>2.2519999999999998</v>
-      </c>
-      <c r="E7" s="7">
-        <f>ROUND(C7-D7,3)</f>
-        <v>0</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
+      <c r="D7" s="5" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="14.4" thickBot="1">
       <c r="A8" s="5" t="s">
         <v>9</v>
       </c>
@@ -55508,15 +55478,8 @@
         <f>B8/1048576</f>
         <v>5240.691837310791</v>
       </c>
-      <c r="D8" s="7">
-        <v>5240.692</v>
-      </c>
-      <c r="E8" s="7">
-        <f>ROUND(C8-D8,3)</f>
-        <v>0</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>250</v>
+      <c r="D8" s="5" t="s">
+        <v>248</v>
       </c>
     </row>
   </sheetData>

</xml_diff>